<commit_message>
Add DOW 3-radio support in gen_html.py and update data files
- gen_html.py: DOW UnitName → 3 radio buttons (CLOSE/OPEN/PAUSE) on single line
- Updated xlsx/json data files with latest SmartFarm tag definitions

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DoForSpring.xlsx
+++ b/DoForSpring.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ClaudeCode\박태영3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35352B87-7BFB-41C4-ADEC-FDC01533B0A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A961A5B0-FF53-4533-84FF-C83E510AB8C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4575" yWindow="1455" windowWidth="21600" windowHeight="11220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tags" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="50">
   <si>
     <t>TagCategory</t>
   </si>
@@ -43,12 +43,27 @@
     <t>OffMsg</t>
   </si>
   <si>
+    <t>양액</t>
+  </si>
+  <si>
+    <t>양액기기동</t>
+  </si>
+  <si>
+    <t>시작정지</t>
+  </si>
+  <si>
     <t>NORMAL</t>
   </si>
   <si>
+    <t>시작</t>
+  </si>
+  <si>
     <t>정지</t>
   </si>
   <si>
+    <t>운전모드</t>
+  </si>
+  <si>
     <t>양액기모드</t>
   </si>
   <si>
@@ -61,37 +76,101 @@
     <t>기본</t>
   </si>
   <si>
+    <t>교반기기동</t>
+  </si>
+  <si>
     <t>교반기</t>
   </si>
   <si>
     <t>교반기모드</t>
   </si>
   <si>
-    <t>양액</t>
+    <t>에어포그</t>
+  </si>
+  <si>
+    <t>포그기동</t>
+  </si>
+  <si>
+    <t>가동</t>
+  </si>
+  <si>
+    <t>포그모드</t>
+  </si>
+  <si>
+    <t>원수펌프기동</t>
+  </si>
+  <si>
+    <t>에어포그원수펌프</t>
+  </si>
+  <si>
+    <t>개폐기</t>
+  </si>
+  <si>
+    <t>천창</t>
+  </si>
+  <si>
+    <t>열림닫힘</t>
+  </si>
+  <si>
+    <t>DOW</t>
+  </si>
+  <si>
+    <t>커튼1</t>
+  </si>
+  <si>
+    <t>커튼2</t>
+  </si>
+  <si>
+    <t>차광막</t>
+  </si>
+  <si>
+    <t>구동기</t>
+  </si>
+  <si>
+    <t>환풍기</t>
+  </si>
+  <si>
+    <t>켜짐</t>
+  </si>
+  <si>
+    <t>꺼짐</t>
+  </si>
+  <si>
+    <t>유동팬</t>
+  </si>
+  <si>
+    <t>훈증기</t>
+  </si>
+  <si>
+    <t>CO2발생기1</t>
+  </si>
+  <si>
+    <t>CO2발생기2</t>
+  </si>
+  <si>
+    <t>보광기</t>
+  </si>
+  <si>
+    <t>보광기1</t>
+  </si>
+  <si>
+    <t>커기끄기</t>
+  </si>
+  <si>
+    <t>보광기2</t>
+  </si>
+  <si>
+    <t>켜기끄기</t>
+  </si>
+  <si>
+    <t>보광기3</t>
+  </si>
+  <si>
+    <t>열기</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>시작정지</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>시작</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>양액기운전모드</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>교반기모드</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>양액기기동</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>교반기기동</t>
+    <t>닫기</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -501,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -534,94 +613,439 @@
     </row>
     <row r="2" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2">
         <v>0</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="E3" s="3">
         <v>1</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E4" s="2">
         <v>16</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="E5" s="3">
         <v>17</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="2">
+        <v>32</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="3">
+        <v>33</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2">
         <v>11</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="F8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="3">
+        <v>48</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="2">
+        <v>50</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="3">
+        <v>52</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="2">
+        <v>54</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" s="3">
+        <v>64</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2">
+        <v>65</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="2">
+        <v>71</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="3">
+        <v>66</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="2">
+        <v>67</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="3">
+        <v>68</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="2">
+        <v>69</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" s="3">
+        <v>70</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>